<commit_message>
Expand optional variables with real registry.chem findings
Replace placeholder optional variables with actual variables found in
Registry/registry.chem that have no history output flag ('h'):
- EDUST1-5: accumulated dust emissions per bin (kg m-2)
- dustload_1-5: dust column loading per bin (ug m-2)
- dustdrydep_1-5: accumulated dust dry deposition (kg m-2)
- dustwdload_1-5: dust wet deposition loss per bin (ug m-2)
- EXTCOF3/106/3_5/8_12: extinction coefficients at other wavelengths
- BSCOF3/106, ASYMPAR3/55/106: backscatter and asymmetry parameters
- PM2_5_EC_DRY, PM2_5_WATER: PM composition diagnostics
- ddflx/wdflx: dry/wet deposition fluxes
- ebu_*: biomass burning emissions
- tropo_p/z: tropopause pressure and height
Total: 440 variables (43 optional, sourced from Registry/registry.chem)

https://claude.ai/code/session_01PqH5Wggp8PGufzqy48e9zR
</commit_message>
<xml_diff>
--- a/wrfout_variables.xlsx
+++ b/wrfout_variables.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Variables'!$A$1:$F$417</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Variables'!$A$1:$F$441</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F417"/>
+  <dimension ref="A1:F441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12155,22 +12155,22 @@
       </c>
       <c r="B399" s="9" t="inlineStr">
         <is>
-          <t>dust_1</t>
+          <t>EDUST1</t>
         </is>
       </c>
       <c r="C399" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D399" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dust bin 1 (0.1-1 um) mixing ratio</t>
+          <t>Accumulated dust emission bin 1 (0.1-1 um)</t>
         </is>
       </c>
       <c r="E399" s="8" t="inlineStr">
         <is>
-          <t>ug/kg-dryair</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F399" s="8" t="inlineStr">
@@ -12185,22 +12185,22 @@
       </c>
       <c r="B400" s="9" t="inlineStr">
         <is>
-          <t>dust_2</t>
+          <t>EDUST2</t>
         </is>
       </c>
       <c r="C400" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D400" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dust bin 2 (1-2.5 um) mixing ratio</t>
+          <t>Accumulated dust emission bin 2 (1-2.5 um)</t>
         </is>
       </c>
       <c r="E400" s="8" t="inlineStr">
         <is>
-          <t>ug/kg-dryair</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F400" s="8" t="inlineStr">
@@ -12215,22 +12215,22 @@
       </c>
       <c r="B401" s="9" t="inlineStr">
         <is>
-          <t>dust_3</t>
+          <t>EDUST3</t>
         </is>
       </c>
       <c r="C401" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D401" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dust bin 3 (2.5-5 um) mixing ratio</t>
+          <t>Accumulated dust emission bin 3 (2.5-5 um)</t>
         </is>
       </c>
       <c r="E401" s="8" t="inlineStr">
         <is>
-          <t>ug/kg-dryair</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F401" s="8" t="inlineStr">
@@ -12245,22 +12245,22 @@
       </c>
       <c r="B402" s="9" t="inlineStr">
         <is>
-          <t>dust_4</t>
+          <t>EDUST4</t>
         </is>
       </c>
       <c r="C402" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D402" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dust bin 4 (5-10 um) mixing ratio</t>
+          <t>Accumulated dust emission bin 4 (5-10 um)</t>
         </is>
       </c>
       <c r="E402" s="8" t="inlineStr">
         <is>
-          <t>ug/kg-dryair</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F402" s="8" t="inlineStr">
@@ -12275,22 +12275,22 @@
       </c>
       <c r="B403" s="9" t="inlineStr">
         <is>
-          <t>dust_5</t>
+          <t>EDUST5</t>
         </is>
       </c>
       <c r="C403" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D403" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dust bin 5 (10-20 um) mixing ratio</t>
+          <t>Accumulated dust emission bin 5 (10-20 um)</t>
         </is>
       </c>
       <c r="E403" s="8" t="inlineStr">
         <is>
-          <t>ug/kg-dryair</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F403" s="8" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="B404" s="9" t="inlineStr">
         <is>
-          <t>DDVEL</t>
+          <t>dustload_1</t>
         </is>
       </c>
       <c r="C404" s="9" t="inlineStr">
@@ -12315,12 +12315,12 @@
       </c>
       <c r="D404" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Dry deposition velocity per species</t>
+          <t>Dust column loading bin 1</t>
         </is>
       </c>
       <c r="E404" s="8" t="inlineStr">
         <is>
-          <t>cm/s</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F404" s="8" t="inlineStr">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="B405" s="9" t="inlineStr">
         <is>
-          <t>wetdep_1</t>
+          <t>dustload_2</t>
         </is>
       </c>
       <c r="C405" s="9" t="inlineStr">
@@ -12345,12 +12345,12 @@
       </c>
       <c r="D405" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Wet deposition flux species 1</t>
+          <t>Dust column loading bin 2</t>
         </is>
       </c>
       <c r="E405" s="8" t="inlineStr">
         <is>
-          <t>mol/km2/hr</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F405" s="8" t="inlineStr">
@@ -12365,22 +12365,22 @@
       </c>
       <c r="B406" s="9" t="inlineStr">
         <is>
-          <t>PHOTR</t>
+          <t>dustload_3</t>
         </is>
       </c>
       <c r="C406" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D406" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Full photolysis rate table (all rates)</t>
+          <t>Dust column loading bin 3</t>
         </is>
       </c>
       <c r="E406" s="8" t="inlineStr">
         <is>
-          <t>min-1</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F406" s="8" t="inlineStr">
@@ -12395,7 +12395,7 @@
       </c>
       <c r="B407" s="9" t="inlineStr">
         <is>
-          <t>ETOT</t>
+          <t>dustload_4</t>
         </is>
       </c>
       <c r="C407" s="9" t="inlineStr">
@@ -12405,12 +12405,12 @@
       </c>
       <c r="D407" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Total anthropogenic emission flux</t>
+          <t>Dust column loading bin 4</t>
         </is>
       </c>
       <c r="E407" s="8" t="inlineStr">
         <is>
-          <t>mol km^-2 hr^-1</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F407" s="8" t="inlineStr">
@@ -12425,7 +12425,7 @@
       </c>
       <c r="B408" s="9" t="inlineStr">
         <is>
-          <t>EBIO</t>
+          <t>dustload_5</t>
         </is>
       </c>
       <c r="C408" s="9" t="inlineStr">
@@ -12435,12 +12435,12 @@
       </c>
       <c r="D408" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Total biogenic emission flux</t>
+          <t>Dust column loading bin 5</t>
         </is>
       </c>
       <c r="E408" s="8" t="inlineStr">
         <is>
-          <t>mol km^-2 hr^-1</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F408" s="8" t="inlineStr">
@@ -12455,7 +12455,7 @@
       </c>
       <c r="B409" s="9" t="inlineStr">
         <is>
-          <t>RAINNCV</t>
+          <t>dustdrydep_1</t>
         </is>
       </c>
       <c r="C409" s="9" t="inlineStr">
@@ -12465,12 +12465,12 @@
       </c>
       <c r="D409" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] TIME-STEP NONCONVECTIVE PRECIPITATION (not in history by default)</t>
+          <t>Accumulated dust dry deposition bin 1</t>
         </is>
       </c>
       <c r="E409" s="8" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F409" s="8" t="inlineStr">
@@ -12485,7 +12485,7 @@
       </c>
       <c r="B410" s="9" t="inlineStr">
         <is>
-          <t>PREC_ACC_NC</t>
+          <t>dustdrydep_2</t>
         </is>
       </c>
       <c r="C410" s="9" t="inlineStr">
@@ -12495,12 +12495,12 @@
       </c>
       <c r="D410" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Accumulated precipitation over interval (requires PREC_ACC_DT)</t>
+          <t>Accumulated dust dry deposition bin 2</t>
         </is>
       </c>
       <c r="E410" s="8" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F410" s="8" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="B411" s="9" t="inlineStr">
         <is>
-          <t>W_UP_MAX</t>
+          <t>dustdrydep_3</t>
         </is>
       </c>
       <c r="C411" s="9" t="inlineStr">
@@ -12525,12 +12525,12 @@
       </c>
       <c r="D411" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Max updraft vertical velocity</t>
+          <t>Accumulated dust dry deposition bin 3</t>
         </is>
       </c>
       <c r="E411" s="8" t="inlineStr">
         <is>
-          <t>m s-1</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F411" s="8" t="inlineStr">
@@ -12545,7 +12545,7 @@
       </c>
       <c r="B412" s="9" t="inlineStr">
         <is>
-          <t>W_DN_MAX</t>
+          <t>dustdrydep_4</t>
         </is>
       </c>
       <c r="C412" s="9" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="D412" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Max downdraft vertical velocity</t>
+          <t>Accumulated dust dry deposition bin 4</t>
         </is>
       </c>
       <c r="E412" s="8" t="inlineStr">
         <is>
-          <t>m s-1</t>
+          <t>kg m-2</t>
         </is>
       </c>
       <c r="F412" s="8" t="inlineStr">
@@ -12575,20 +12575,24 @@
       </c>
       <c r="B413" s="9" t="inlineStr">
         <is>
-          <t>CLDFRA_CONV</t>
+          <t>dustdrydep_5</t>
         </is>
       </c>
       <c r="C413" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D413" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Convective cloud fraction</t>
-        </is>
-      </c>
-      <c r="E413" s="8" t="inlineStr"/>
+          <t>Accumulated dust dry deposition bin 5</t>
+        </is>
+      </c>
+      <c r="E413" s="8" t="inlineStr">
+        <is>
+          <t>kg m-2</t>
+        </is>
+      </c>
       <c r="F413" s="8" t="inlineStr">
         <is>
           <t>Can be added</t>
@@ -12601,7 +12605,7 @@
       </c>
       <c r="B414" s="9" t="inlineStr">
         <is>
-          <t>ACHEMS_DRY</t>
+          <t>dustwdload_1</t>
         </is>
       </c>
       <c r="C414" s="9" t="inlineStr">
@@ -12611,12 +12615,12 @@
       </c>
       <c r="D414" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Accumulated dry deposition per species</t>
+          <t>Dust load loss by wet deposition bin 1</t>
         </is>
       </c>
       <c r="E414" s="8" t="inlineStr">
         <is>
-          <t>mol km^-2</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F414" s="8" t="inlineStr">
@@ -12631,7 +12635,7 @@
       </c>
       <c r="B415" s="9" t="inlineStr">
         <is>
-          <t>ACHEMS_WET</t>
+          <t>dustwdload_2</t>
         </is>
       </c>
       <c r="C415" s="9" t="inlineStr">
@@ -12641,12 +12645,12 @@
       </c>
       <c r="D415" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Accumulated wet deposition per species</t>
+          <t>Dust load loss by wet deposition bin 2</t>
         </is>
       </c>
       <c r="E415" s="8" t="inlineStr">
         <is>
-          <t>mol km^-2</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F415" s="8" t="inlineStr">
@@ -12661,22 +12665,22 @@
       </c>
       <c r="B416" s="9" t="inlineStr">
         <is>
-          <t>den</t>
+          <t>dustwdload_3</t>
         </is>
       </c>
       <c r="C416" s="9" t="inlineStr">
         <is>
-          <t>Time, bottom_top, south_north, west_east</t>
+          <t>Time, south_north, west_east</t>
         </is>
       </c>
       <c r="D416" s="9" t="inlineStr">
         <is>
-          <t>[OPTIONAL] Air density (computed, not output by default)</t>
+          <t>Dust load loss by wet deposition bin 3</t>
         </is>
       </c>
       <c r="E416" s="8" t="inlineStr">
         <is>
-          <t>kg m^-3</t>
+          <t>ug m-2</t>
         </is>
       </c>
       <c r="F416" s="8" t="inlineStr">
@@ -12691,32 +12695,740 @@
       </c>
       <c r="B417" s="9" t="inlineStr">
         <is>
+          <t>dustwdload_4</t>
+        </is>
+      </c>
+      <c r="C417" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D417" s="9" t="inlineStr">
+        <is>
+          <t>Dust load loss by wet deposition bin 4</t>
+        </is>
+      </c>
+      <c r="E417" s="8" t="inlineStr">
+        <is>
+          <t>ug m-2</t>
+        </is>
+      </c>
+      <c r="F417" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="418" ht="18" customHeight="1">
+      <c r="A418" s="8" t="n">
+        <v>417</v>
+      </c>
+      <c r="B418" s="9" t="inlineStr">
+        <is>
+          <t>dustwdload_5</t>
+        </is>
+      </c>
+      <c r="C418" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D418" s="9" t="inlineStr">
+        <is>
+          <t>Dust load loss by wet deposition bin 5</t>
+        </is>
+      </c>
+      <c r="E418" s="8" t="inlineStr">
+        <is>
+          <t>ug m-2</t>
+        </is>
+      </c>
+      <c r="F418" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="419" ht="18" customHeight="1">
+      <c r="A419" s="8" t="n">
+        <v>418</v>
+      </c>
+      <c r="B419" s="9" t="inlineStr">
+        <is>
+          <t>EXTCOF3</t>
+        </is>
+      </c>
+      <c r="C419" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D419" s="9" t="inlineStr">
+        <is>
+          <t>Extinction coefficient at 0.3 um</t>
+        </is>
+      </c>
+      <c r="E419" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F419" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="420" ht="18" customHeight="1">
+      <c r="A420" s="8" t="n">
+        <v>419</v>
+      </c>
+      <c r="B420" s="9" t="inlineStr">
+        <is>
+          <t>EXTCOF106</t>
+        </is>
+      </c>
+      <c r="C420" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D420" s="9" t="inlineStr">
+        <is>
+          <t>Extinction coefficient at 1.06 um</t>
+        </is>
+      </c>
+      <c r="E420" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F420" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="421" ht="18" customHeight="1">
+      <c r="A421" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="B421" s="9" t="inlineStr">
+        <is>
+          <t>EXTCOF3_5</t>
+        </is>
+      </c>
+      <c r="C421" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D421" s="9" t="inlineStr">
+        <is>
+          <t>Band-avg extinction 3-5 um</t>
+        </is>
+      </c>
+      <c r="E421" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F421" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="422" ht="18" customHeight="1">
+      <c r="A422" s="8" t="n">
+        <v>421</v>
+      </c>
+      <c r="B422" s="9" t="inlineStr">
+        <is>
+          <t>EXTCOF8_12</t>
+        </is>
+      </c>
+      <c r="C422" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D422" s="9" t="inlineStr">
+        <is>
+          <t>Band-avg extinction 8-12 um</t>
+        </is>
+      </c>
+      <c r="E422" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F422" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="423" ht="18" customHeight="1">
+      <c r="A423" s="8" t="n">
+        <v>422</v>
+      </c>
+      <c r="B423" s="9" t="inlineStr">
+        <is>
+          <t>BSCOF3</t>
+        </is>
+      </c>
+      <c r="C423" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D423" s="9" t="inlineStr">
+        <is>
+          <t>Backscatter coefficient at 0.3 um</t>
+        </is>
+      </c>
+      <c r="E423" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F423" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="424" ht="18" customHeight="1">
+      <c r="A424" s="8" t="n">
+        <v>423</v>
+      </c>
+      <c r="B424" s="9" t="inlineStr">
+        <is>
+          <t>BSCOF106</t>
+        </is>
+      </c>
+      <c r="C424" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D424" s="9" t="inlineStr">
+        <is>
+          <t>Backscatter coefficient at 1.06 um</t>
+        </is>
+      </c>
+      <c r="E424" s="8" t="inlineStr">
+        <is>
+          <t>km-1</t>
+        </is>
+      </c>
+      <c r="F424" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="425" ht="18" customHeight="1">
+      <c r="A425" s="8" t="n">
+        <v>424</v>
+      </c>
+      <c r="B425" s="9" t="inlineStr">
+        <is>
+          <t>ASYMPAR3</t>
+        </is>
+      </c>
+      <c r="C425" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D425" s="9" t="inlineStr">
+        <is>
+          <t>Asymmetry parameter at 0.3 um</t>
+        </is>
+      </c>
+      <c r="E425" s="8" t="inlineStr"/>
+      <c r="F425" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="426" ht="18" customHeight="1">
+      <c r="A426" s="8" t="n">
+        <v>425</v>
+      </c>
+      <c r="B426" s="9" t="inlineStr">
+        <is>
+          <t>ASYMPAR55</t>
+        </is>
+      </c>
+      <c r="C426" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D426" s="9" t="inlineStr">
+        <is>
+          <t>Asymmetry parameter at 0.55 um</t>
+        </is>
+      </c>
+      <c r="E426" s="8" t="inlineStr"/>
+      <c r="F426" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="427" ht="18" customHeight="1">
+      <c r="A427" s="8" t="n">
+        <v>426</v>
+      </c>
+      <c r="B427" s="9" t="inlineStr">
+        <is>
+          <t>ASYMPAR106</t>
+        </is>
+      </c>
+      <c r="C427" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D427" s="9" t="inlineStr">
+        <is>
+          <t>Asymmetry parameter at 1.06 um</t>
+        </is>
+      </c>
+      <c r="E427" s="8" t="inlineStr"/>
+      <c r="F427" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="428" ht="18" customHeight="1">
+      <c r="A428" s="8" t="n">
+        <v>427</v>
+      </c>
+      <c r="B428" s="9" t="inlineStr">
+        <is>
+          <t>PM2_5_EC_DRY</t>
+        </is>
+      </c>
+      <c r="C428" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D428" s="9" t="inlineStr">
+        <is>
+          <t>PM2.5 elemental carbon dry mass</t>
+        </is>
+      </c>
+      <c r="E428" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F428" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="429" ht="18" customHeight="1">
+      <c r="A429" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="B429" s="9" t="inlineStr">
+        <is>
+          <t>PM2_5_WATER</t>
+        </is>
+      </c>
+      <c r="C429" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D429" s="9" t="inlineStr">
+        <is>
+          <t>PM2.5 aerosol liquid water content</t>
+        </is>
+      </c>
+      <c r="E429" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F429" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="430" ht="18" customHeight="1">
+      <c r="A430" s="8" t="n">
+        <v>429</v>
+      </c>
+      <c r="B430" s="9" t="inlineStr">
+        <is>
+          <t>ddflx</t>
+        </is>
+      </c>
+      <c r="C430" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D430" s="9" t="inlineStr">
+        <is>
+          <t>Dry deposition flux for chemical species</t>
+        </is>
+      </c>
+      <c r="E430" s="8" t="inlineStr">
+        <is>
+          <t>mol m-2 or ug m-2</t>
+        </is>
+      </c>
+      <c r="F430" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="431" ht="18" customHeight="1">
+      <c r="A431" s="8" t="n">
+        <v>430</v>
+      </c>
+      <c r="B431" s="9" t="inlineStr">
+        <is>
+          <t>wdflx</t>
+        </is>
+      </c>
+      <c r="C431" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D431" s="9" t="inlineStr">
+        <is>
+          <t>Column wet scavenging flux for species</t>
+        </is>
+      </c>
+      <c r="E431" s="8" t="inlineStr">
+        <is>
+          <t>mmol m-2 or ug m-2</t>
+        </is>
+      </c>
+      <c r="F431" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="432" ht="18" customHeight="1">
+      <c r="A432" s="8" t="n">
+        <v>431</v>
+      </c>
+      <c r="B432" s="9" t="inlineStr">
+        <is>
+          <t>ebu_pm25</t>
+        </is>
+      </c>
+      <c r="C432" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D432" s="9" t="inlineStr">
+        <is>
+          <t>PM2.5 from biomass burning</t>
+        </is>
+      </c>
+      <c r="E432" s="8" t="inlineStr">
+        <is>
+          <t>ug m-2 s-1</t>
+        </is>
+      </c>
+      <c r="F432" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="433" ht="18" customHeight="1">
+      <c r="A433" s="8" t="n">
+        <v>432</v>
+      </c>
+      <c r="B433" s="9" t="inlineStr">
+        <is>
+          <t>ebu_pm10</t>
+        </is>
+      </c>
+      <c r="C433" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D433" s="9" t="inlineStr">
+        <is>
+          <t>PM10 from biomass burning</t>
+        </is>
+      </c>
+      <c r="E433" s="8" t="inlineStr">
+        <is>
+          <t>ug m-2 s-1</t>
+        </is>
+      </c>
+      <c r="F433" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="434" ht="18" customHeight="1">
+      <c r="A434" s="8" t="n">
+        <v>433</v>
+      </c>
+      <c r="B434" s="9" t="inlineStr">
+        <is>
+          <t>ebu_bc</t>
+        </is>
+      </c>
+      <c r="C434" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D434" s="9" t="inlineStr">
+        <is>
+          <t>Black carbon from biomass burning</t>
+        </is>
+      </c>
+      <c r="E434" s="8" t="inlineStr">
+        <is>
+          <t>ug m-2 s-1</t>
+        </is>
+      </c>
+      <c r="F434" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="435" ht="18" customHeight="1">
+      <c r="A435" s="8" t="n">
+        <v>434</v>
+      </c>
+      <c r="B435" s="9" t="inlineStr">
+        <is>
+          <t>ebu_co</t>
+        </is>
+      </c>
+      <c r="C435" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D435" s="9" t="inlineStr">
+        <is>
+          <t>CO from biomass burning</t>
+        </is>
+      </c>
+      <c r="E435" s="8" t="inlineStr">
+        <is>
+          <t>mol km-2 hr-1</t>
+        </is>
+      </c>
+      <c r="F435" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="436" ht="18" customHeight="1">
+      <c r="A436" s="8" t="n">
+        <v>435</v>
+      </c>
+      <c r="B436" s="9" t="inlineStr">
+        <is>
+          <t>tropo_p</t>
+        </is>
+      </c>
+      <c r="C436" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D436" s="9" t="inlineStr">
+        <is>
+          <t>Tropopause pressure</t>
+        </is>
+      </c>
+      <c r="E436" s="8" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="F436" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="437" ht="18" customHeight="1">
+      <c r="A437" s="8" t="n">
+        <v>436</v>
+      </c>
+      <c r="B437" s="9" t="inlineStr">
+        <is>
+          <t>tropo_z</t>
+        </is>
+      </c>
+      <c r="C437" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D437" s="9" t="inlineStr">
+        <is>
+          <t>Tropopause height</t>
+        </is>
+      </c>
+      <c r="E437" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F437" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="438" ht="18" customHeight="1">
+      <c r="A438" s="8" t="n">
+        <v>437</v>
+      </c>
+      <c r="B438" s="9" t="inlineStr">
+        <is>
+          <t>RAINNCV</t>
+        </is>
+      </c>
+      <c r="C438" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D438" s="9" t="inlineStr">
+        <is>
+          <t>TIME-STEP NONCONVECTIVE PRECIPITATION (restart only, not history)</t>
+        </is>
+      </c>
+      <c r="E438" s="8" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F438" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="439" ht="18" customHeight="1">
+      <c r="A439" s="8" t="n">
+        <v>438</v>
+      </c>
+      <c r="B439" s="9" t="inlineStr">
+        <is>
+          <t>PREC_ACC_NC</t>
+        </is>
+      </c>
+      <c r="C439" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D439" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated precip over interval (requires PREC_ACC_DT &gt; 0 in namelist)</t>
+        </is>
+      </c>
+      <c r="E439" s="8" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F439" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="440" ht="18" customHeight="1">
+      <c r="A440" s="8" t="n">
+        <v>439</v>
+      </c>
+      <c r="B440" s="9" t="inlineStr">
+        <is>
+          <t>den</t>
+        </is>
+      </c>
+      <c r="C440" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D440" s="9" t="inlineStr">
+        <is>
+          <t>Air density (computed internally, not output by default)</t>
+        </is>
+      </c>
+      <c r="E440" s="8" t="inlineStr">
+        <is>
+          <t>kg m-3</t>
+        </is>
+      </c>
+      <c r="F440" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="441" ht="18" customHeight="1">
+      <c r="A441" s="8" t="n">
+        <v>440</v>
+      </c>
+      <c r="B441" s="9" t="inlineStr">
+        <is>
           <t>alt</t>
         </is>
       </c>
-      <c r="C417" s="9" t="inlineStr">
-        <is>
-          <t>Time, bottom_top, south_north, west_east</t>
-        </is>
-      </c>
-      <c r="D417" s="9" t="inlineStr">
-        <is>
-          <t>[OPTIONAL] Inverse density (specific volume)</t>
-        </is>
-      </c>
-      <c r="E417" s="8" t="inlineStr">
+      <c r="C441" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D441" s="9" t="inlineStr">
+        <is>
+          <t>Inverse density / specific volume (not output by default)</t>
+        </is>
+      </c>
+      <c r="E441" s="8" t="inlineStr">
         <is>
           <t>m3 kg-1</t>
         </is>
       </c>
-      <c r="F417" s="8" t="inlineStr">
+      <c r="F441" s="8" t="inlineStr">
         <is>
           <t>Can be added</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F417"/>
+  <autoFilter ref="A1:F441"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add more optional variables from registry.chem deep search
Additional verified variables from Registry/registry.chem:
- dustwd_1-5: 3D dust wet deposition loss (ug/kg-dryair)
- chem_co/o3/no/no2/hno3/ho/ho2: chemical tendency diagnostics (enable: chemdiag=1)
- hoa_a01, soa_a01, bboa_a01, bbsoa_a01, totoa_a01: aerosol OC breakdown (aero_diag_opt=1)
- sulf_srf_area, oc_srf_area, bc_srf_area: aerosol surface area (aero_srf_area_diag=1)
- ph_aer01-04: aerosol bin H+ concentration (mol/kg)
- af_dir/up/dn: actinic flux components (W m-2 nm-1)
- dvel_no2/nh3/hno3/so2: deposition velocities for key gases
Total: 471 variables (74 optional)

https://claude.ai/code/session_01PqH5Wggp8PGufzqy48e9zR
</commit_message>
<xml_diff>
--- a/wrfout_variables.xlsx
+++ b/wrfout_variables.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Variables'!$A$1:$F$441</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Variables'!$A$1:$F$472</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F441"/>
+  <dimension ref="A1:F472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13313,22 +13313,22 @@
       </c>
       <c r="B438" s="9" t="inlineStr">
         <is>
-          <t>RAINNCV</t>
+          <t>dustwd_1</t>
         </is>
       </c>
       <c r="C438" s="9" t="inlineStr">
         <is>
-          <t>Time, south_north, west_east</t>
+          <t>Time, bottom_top, south_north, west_east</t>
         </is>
       </c>
       <c r="D438" s="9" t="inlineStr">
         <is>
-          <t>TIME-STEP NONCONVECTIVE PRECIPITATION (restart only, not history)</t>
+          <t>Dust loss by wet deposition bin 1</t>
         </is>
       </c>
       <c r="E438" s="8" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>ug/kg-dryair</t>
         </is>
       </c>
       <c r="F438" s="8" t="inlineStr">
@@ -13343,22 +13343,22 @@
       </c>
       <c r="B439" s="9" t="inlineStr">
         <is>
-          <t>PREC_ACC_NC</t>
+          <t>dustwd_2</t>
         </is>
       </c>
       <c r="C439" s="9" t="inlineStr">
         <is>
-          <t>Time, south_north, west_east</t>
+          <t>Time, bottom_top, south_north, west_east</t>
         </is>
       </c>
       <c r="D439" s="9" t="inlineStr">
         <is>
-          <t>Accumulated precip over interval (requires PREC_ACC_DT &gt; 0 in namelist)</t>
+          <t>Dust loss by wet deposition bin 2</t>
         </is>
       </c>
       <c r="E439" s="8" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>ug/kg-dryair</t>
         </is>
       </c>
       <c r="F439" s="8" t="inlineStr">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="B440" s="9" t="inlineStr">
         <is>
-          <t>den</t>
+          <t>dustwd_3</t>
         </is>
       </c>
       <c r="C440" s="9" t="inlineStr">
@@ -13383,12 +13383,12 @@
       </c>
       <c r="D440" s="9" t="inlineStr">
         <is>
-          <t>Air density (computed internally, not output by default)</t>
+          <t>Dust loss by wet deposition bin 3</t>
         </is>
       </c>
       <c r="E440" s="8" t="inlineStr">
         <is>
-          <t>kg m-3</t>
+          <t>ug/kg-dryair</t>
         </is>
       </c>
       <c r="F440" s="8" t="inlineStr">
@@ -13403,32 +13403,962 @@
       </c>
       <c r="B441" s="9" t="inlineStr">
         <is>
+          <t>dustwd_4</t>
+        </is>
+      </c>
+      <c r="C441" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D441" s="9" t="inlineStr">
+        <is>
+          <t>Dust loss by wet deposition bin 4</t>
+        </is>
+      </c>
+      <c r="E441" s="8" t="inlineStr">
+        <is>
+          <t>ug/kg-dryair</t>
+        </is>
+      </c>
+      <c r="F441" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="442" ht="18" customHeight="1">
+      <c r="A442" s="8" t="n">
+        <v>441</v>
+      </c>
+      <c r="B442" s="9" t="inlineStr">
+        <is>
+          <t>dustwd_5</t>
+        </is>
+      </c>
+      <c r="C442" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D442" s="9" t="inlineStr">
+        <is>
+          <t>Dust loss by wet deposition bin 5</t>
+        </is>
+      </c>
+      <c r="E442" s="8" t="inlineStr">
+        <is>
+          <t>ug/kg-dryair</t>
+        </is>
+      </c>
+      <c r="F442" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="443" ht="18" customHeight="1">
+      <c r="A443" s="8" t="n">
+        <v>442</v>
+      </c>
+      <c r="B443" s="9" t="inlineStr">
+        <is>
+          <t>chem_co</t>
+        </is>
+      </c>
+      <c r="C443" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D443" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for CO  [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E443" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F443" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="444" ht="18" customHeight="1">
+      <c r="A444" s="8" t="n">
+        <v>443</v>
+      </c>
+      <c r="B444" s="9" t="inlineStr">
+        <is>
+          <t>chem_o3</t>
+        </is>
+      </c>
+      <c r="C444" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D444" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for O3  [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E444" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F444" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="445" ht="18" customHeight="1">
+      <c r="A445" s="8" t="n">
+        <v>444</v>
+      </c>
+      <c r="B445" s="9" t="inlineStr">
+        <is>
+          <t>chem_no</t>
+        </is>
+      </c>
+      <c r="C445" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D445" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for NO  [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E445" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F445" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="446" ht="18" customHeight="1">
+      <c r="A446" s="8" t="n">
+        <v>445</v>
+      </c>
+      <c r="B446" s="9" t="inlineStr">
+        <is>
+          <t>chem_no2</t>
+        </is>
+      </c>
+      <c r="C446" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D446" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for NO2 [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E446" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F446" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="447" ht="18" customHeight="1">
+      <c r="A447" s="8" t="n">
+        <v>446</v>
+      </c>
+      <c r="B447" s="9" t="inlineStr">
+        <is>
+          <t>chem_hno3</t>
+        </is>
+      </c>
+      <c r="C447" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D447" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for HNO3 [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E447" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F447" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="448" ht="18" customHeight="1">
+      <c r="A448" s="8" t="n">
+        <v>447</v>
+      </c>
+      <c r="B448" s="9" t="inlineStr">
+        <is>
+          <t>chem_ho</t>
+        </is>
+      </c>
+      <c r="C448" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D448" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for HO  [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E448" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F448" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="449" ht="18" customHeight="1">
+      <c r="A449" s="8" t="n">
+        <v>448</v>
+      </c>
+      <c r="B449" s="9" t="inlineStr">
+        <is>
+          <t>chem_ho2</t>
+        </is>
+      </c>
+      <c r="C449" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D449" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated chemical tendency for HO2 [chemdiag=1]</t>
+        </is>
+      </c>
+      <c r="E449" s="8" t="inlineStr">
+        <is>
+          <t>ppmv</t>
+        </is>
+      </c>
+      <c r="F449" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="450" ht="18" customHeight="1">
+      <c r="A450" s="8" t="n">
+        <v>449</v>
+      </c>
+      <c r="B450" s="9" t="inlineStr">
+        <is>
+          <t>hoa_a01</t>
+        </is>
+      </c>
+      <c r="C450" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D450" s="9" t="inlineStr">
+        <is>
+          <t>Hydrophobic anthropogenic OA bin 1 [aero_diag_opt=1]</t>
+        </is>
+      </c>
+      <c r="E450" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F450" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="451" ht="18" customHeight="1">
+      <c r="A451" s="8" t="n">
+        <v>450</v>
+      </c>
+      <c r="B451" s="9" t="inlineStr">
+        <is>
+          <t>soa_a01</t>
+        </is>
+      </c>
+      <c r="C451" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D451" s="9" t="inlineStr">
+        <is>
+          <t>Secondary organic aerosol bin 1    [aero_diag_opt=1]</t>
+        </is>
+      </c>
+      <c r="E451" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F451" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="452" ht="18" customHeight="1">
+      <c r="A452" s="8" t="n">
+        <v>451</v>
+      </c>
+      <c r="B452" s="9" t="inlineStr">
+        <is>
+          <t>bboa_a01</t>
+        </is>
+      </c>
+      <c r="C452" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D452" s="9" t="inlineStr">
+        <is>
+          <t>Biomass burning OA bin 1           [aero_diag_opt=1]</t>
+        </is>
+      </c>
+      <c r="E452" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F452" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="453" ht="18" customHeight="1">
+      <c r="A453" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="B453" s="9" t="inlineStr">
+        <is>
+          <t>bbsoa_a01</t>
+        </is>
+      </c>
+      <c r="C453" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D453" s="9" t="inlineStr">
+        <is>
+          <t>Biomass burning SOA bin 1          [aero_diag_opt=1]</t>
+        </is>
+      </c>
+      <c r="E453" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F453" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="454" ht="18" customHeight="1">
+      <c r="A454" s="8" t="n">
+        <v>453</v>
+      </c>
+      <c r="B454" s="9" t="inlineStr">
+        <is>
+          <t>totoa_a01</t>
+        </is>
+      </c>
+      <c r="C454" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D454" s="9" t="inlineStr">
+        <is>
+          <t>Total OA bin 1                     [aero_diag_opt=1]</t>
+        </is>
+      </c>
+      <c r="E454" s="8" t="inlineStr">
+        <is>
+          <t>ug m-3</t>
+        </is>
+      </c>
+      <c r="F454" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="455" ht="18" customHeight="1">
+      <c r="A455" s="8" t="n">
+        <v>454</v>
+      </c>
+      <c r="B455" s="9" t="inlineStr">
+        <is>
+          <t>sulf_srf_area</t>
+        </is>
+      </c>
+      <c r="C455" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D455" s="9" t="inlineStr">
+        <is>
+          <t>Sulfate aerosol surface area  [aero_srf_area_diag=1]</t>
+        </is>
+      </c>
+      <c r="E455" s="8" t="inlineStr">
+        <is>
+          <t>cm2</t>
+        </is>
+      </c>
+      <c r="F455" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="456" ht="18" customHeight="1">
+      <c r="A456" s="8" t="n">
+        <v>455</v>
+      </c>
+      <c r="B456" s="9" t="inlineStr">
+        <is>
+          <t>oc_srf_area</t>
+        </is>
+      </c>
+      <c r="C456" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D456" s="9" t="inlineStr">
+        <is>
+          <t>Hydrophilic OC aerosol surface area [aero_srf_area_diag=1]</t>
+        </is>
+      </c>
+      <c r="E456" s="8" t="inlineStr">
+        <is>
+          <t>cm2</t>
+        </is>
+      </c>
+      <c r="F456" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="457" ht="18" customHeight="1">
+      <c r="A457" s="8" t="n">
+        <v>456</v>
+      </c>
+      <c r="B457" s="9" t="inlineStr">
+        <is>
+          <t>bc_srf_area</t>
+        </is>
+      </c>
+      <c r="C457" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D457" s="9" t="inlineStr">
+        <is>
+          <t>Hydrophilic BC aerosol surface area [aero_srf_area_diag=1]</t>
+        </is>
+      </c>
+      <c r="E457" s="8" t="inlineStr">
+        <is>
+          <t>cm2</t>
+        </is>
+      </c>
+      <c r="F457" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="458" ht="18" customHeight="1">
+      <c r="A458" s="8" t="n">
+        <v>457</v>
+      </c>
+      <c r="B458" s="9" t="inlineStr">
+        <is>
+          <t>ph_aer01</t>
+        </is>
+      </c>
+      <c r="C458" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D458" s="9" t="inlineStr">
+        <is>
+          <t>H+ concentration in aerosol bin 1</t>
+        </is>
+      </c>
+      <c r="E458" s="8" t="inlineStr">
+        <is>
+          <t>mol/kg</t>
+        </is>
+      </c>
+      <c r="F458" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="459" ht="18" customHeight="1">
+      <c r="A459" s="8" t="n">
+        <v>458</v>
+      </c>
+      <c r="B459" s="9" t="inlineStr">
+        <is>
+          <t>ph_aer02</t>
+        </is>
+      </c>
+      <c r="C459" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D459" s="9" t="inlineStr">
+        <is>
+          <t>H+ concentration in aerosol bin 2</t>
+        </is>
+      </c>
+      <c r="E459" s="8" t="inlineStr">
+        <is>
+          <t>mol/kg</t>
+        </is>
+      </c>
+      <c r="F459" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="460" ht="18" customHeight="1">
+      <c r="A460" s="8" t="n">
+        <v>459</v>
+      </c>
+      <c r="B460" s="9" t="inlineStr">
+        <is>
+          <t>ph_aer03</t>
+        </is>
+      </c>
+      <c r="C460" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D460" s="9" t="inlineStr">
+        <is>
+          <t>H+ concentration in aerosol bin 3</t>
+        </is>
+      </c>
+      <c r="E460" s="8" t="inlineStr">
+        <is>
+          <t>mol/kg</t>
+        </is>
+      </c>
+      <c r="F460" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="461" ht="18" customHeight="1">
+      <c r="A461" s="8" t="n">
+        <v>460</v>
+      </c>
+      <c r="B461" s="9" t="inlineStr">
+        <is>
+          <t>ph_aer04</t>
+        </is>
+      </c>
+      <c r="C461" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D461" s="9" t="inlineStr">
+        <is>
+          <t>H+ concentration in aerosol bin 4</t>
+        </is>
+      </c>
+      <c r="E461" s="8" t="inlineStr">
+        <is>
+          <t>mol/kg</t>
+        </is>
+      </c>
+      <c r="F461" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="462" ht="18" customHeight="1">
+      <c r="A462" s="8" t="n">
+        <v>461</v>
+      </c>
+      <c r="B462" s="9" t="inlineStr">
+        <is>
+          <t>af_dir</t>
+        </is>
+      </c>
+      <c r="C462" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D462" s="9" t="inlineStr">
+        <is>
+          <t>Actinic flux direct</t>
+        </is>
+      </c>
+      <c r="E462" s="8" t="inlineStr">
+        <is>
+          <t>W m-2 nm-1</t>
+        </is>
+      </c>
+      <c r="F462" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="18" customHeight="1">
+      <c r="A463" s="8" t="n">
+        <v>462</v>
+      </c>
+      <c r="B463" s="9" t="inlineStr">
+        <is>
+          <t>af_up</t>
+        </is>
+      </c>
+      <c r="C463" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D463" s="9" t="inlineStr">
+        <is>
+          <t>Actinic flux upwelling</t>
+        </is>
+      </c>
+      <c r="E463" s="8" t="inlineStr">
+        <is>
+          <t>W m-2 nm-1</t>
+        </is>
+      </c>
+      <c r="F463" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="464" ht="18" customHeight="1">
+      <c r="A464" s="8" t="n">
+        <v>463</v>
+      </c>
+      <c r="B464" s="9" t="inlineStr">
+        <is>
+          <t>af_dn</t>
+        </is>
+      </c>
+      <c r="C464" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D464" s="9" t="inlineStr">
+        <is>
+          <t>Actinic flux downwelling</t>
+        </is>
+      </c>
+      <c r="E464" s="8" t="inlineStr">
+        <is>
+          <t>W m-2 nm-1</t>
+        </is>
+      </c>
+      <c r="F464" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="465" ht="18" customHeight="1">
+      <c r="A465" s="8" t="n">
+        <v>464</v>
+      </c>
+      <c r="B465" s="9" t="inlineStr">
+        <is>
+          <t>dvel_no2</t>
+        </is>
+      </c>
+      <c r="C465" s="9" t="inlineStr">
+        <is>
+          <t>Time, klevs_for_dvel, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D465" s="9" t="inlineStr">
+        <is>
+          <t>NO2 deposition velocity</t>
+        </is>
+      </c>
+      <c r="E465" s="8" t="inlineStr">
+        <is>
+          <t>cm/s</t>
+        </is>
+      </c>
+      <c r="F465" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="466" ht="18" customHeight="1">
+      <c r="A466" s="8" t="n">
+        <v>465</v>
+      </c>
+      <c r="B466" s="9" t="inlineStr">
+        <is>
+          <t>dvel_nh3</t>
+        </is>
+      </c>
+      <c r="C466" s="9" t="inlineStr">
+        <is>
+          <t>Time, klevs_for_dvel, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D466" s="9" t="inlineStr">
+        <is>
+          <t>NH3 deposition velocity</t>
+        </is>
+      </c>
+      <c r="E466" s="8" t="inlineStr">
+        <is>
+          <t>cm/s</t>
+        </is>
+      </c>
+      <c r="F466" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="467" ht="18" customHeight="1">
+      <c r="A467" s="8" t="n">
+        <v>466</v>
+      </c>
+      <c r="B467" s="9" t="inlineStr">
+        <is>
+          <t>dvel_hno3</t>
+        </is>
+      </c>
+      <c r="C467" s="9" t="inlineStr">
+        <is>
+          <t>Time, klevs_for_dvel, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D467" s="9" t="inlineStr">
+        <is>
+          <t>HNO3 deposition velocity</t>
+        </is>
+      </c>
+      <c r="E467" s="8" t="inlineStr">
+        <is>
+          <t>cm/s</t>
+        </is>
+      </c>
+      <c r="F467" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="468" ht="18" customHeight="1">
+      <c r="A468" s="8" t="n">
+        <v>467</v>
+      </c>
+      <c r="B468" s="9" t="inlineStr">
+        <is>
+          <t>dvel_so2</t>
+        </is>
+      </c>
+      <c r="C468" s="9" t="inlineStr">
+        <is>
+          <t>Time, klevs_for_dvel, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D468" s="9" t="inlineStr">
+        <is>
+          <t>SO2 deposition velocity</t>
+        </is>
+      </c>
+      <c r="E468" s="8" t="inlineStr">
+        <is>
+          <t>cm/s</t>
+        </is>
+      </c>
+      <c r="F468" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="469" ht="18" customHeight="1">
+      <c r="A469" s="8" t="n">
+        <v>468</v>
+      </c>
+      <c r="B469" s="9" t="inlineStr">
+        <is>
+          <t>RAINNCV</t>
+        </is>
+      </c>
+      <c r="C469" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D469" s="9" t="inlineStr">
+        <is>
+          <t>TIME-STEP NONCONVECTIVE PRECIPITATION (restart only, not history)</t>
+        </is>
+      </c>
+      <c r="E469" s="8" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F469" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="18" customHeight="1">
+      <c r="A470" s="8" t="n">
+        <v>469</v>
+      </c>
+      <c r="B470" s="9" t="inlineStr">
+        <is>
+          <t>PREC_ACC_NC</t>
+        </is>
+      </c>
+      <c r="C470" s="9" t="inlineStr">
+        <is>
+          <t>Time, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D470" s="9" t="inlineStr">
+        <is>
+          <t>Accumulated precip over interval (requires PREC_ACC_DT &gt; 0 in namelist)</t>
+        </is>
+      </c>
+      <c r="E470" s="8" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F470" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="471" ht="18" customHeight="1">
+      <c r="A471" s="8" t="n">
+        <v>470</v>
+      </c>
+      <c r="B471" s="9" t="inlineStr">
+        <is>
+          <t>den</t>
+        </is>
+      </c>
+      <c r="C471" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D471" s="9" t="inlineStr">
+        <is>
+          <t>Air density (computed internally, not output by default)</t>
+        </is>
+      </c>
+      <c r="E471" s="8" t="inlineStr">
+        <is>
+          <t>kg m-3</t>
+        </is>
+      </c>
+      <c r="F471" s="8" t="inlineStr">
+        <is>
+          <t>Can be added</t>
+        </is>
+      </c>
+    </row>
+    <row r="472" ht="18" customHeight="1">
+      <c r="A472" s="8" t="n">
+        <v>471</v>
+      </c>
+      <c r="B472" s="9" t="inlineStr">
+        <is>
           <t>alt</t>
         </is>
       </c>
-      <c r="C441" s="9" t="inlineStr">
-        <is>
-          <t>Time, bottom_top, south_north, west_east</t>
-        </is>
-      </c>
-      <c r="D441" s="9" t="inlineStr">
+      <c r="C472" s="9" t="inlineStr">
+        <is>
+          <t>Time, bottom_top, south_north, west_east</t>
+        </is>
+      </c>
+      <c r="D472" s="9" t="inlineStr">
         <is>
           <t>Inverse density / specific volume (not output by default)</t>
         </is>
       </c>
-      <c r="E441" s="8" t="inlineStr">
+      <c r="E472" s="8" t="inlineStr">
         <is>
           <t>m3 kg-1</t>
         </is>
       </c>
-      <c r="F441" s="8" t="inlineStr">
+      <c r="F472" s="8" t="inlineStr">
         <is>
           <t>Can be added</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F441"/>
+  <autoFilter ref="A1:F472"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>